<commit_message>
added updated settings for officer
</commit_message>
<xml_diff>
--- a/public/students-template.xlsx
+++ b/public/students-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5F9F88AD-BDCE-41D8-95CC-DC66418599D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{362DE447-BA26-4921-9523-647B259D4345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{B955C56F-2064-49CD-8B61-0960BC06AA2A}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>name</t>
   </si>
@@ -56,13 +56,37 @@
   </si>
   <si>
     <t>plustwo_streams</t>
+  </si>
+  <si>
+    <t>Mohammed Shuhaib M</t>
+  </si>
+  <si>
+    <t>AL-4</t>
+  </si>
+  <si>
+    <t>INSHIRAH</t>
+  </si>
+  <si>
+    <t>Batch 12</t>
+  </si>
+  <si>
+    <t>Muneer S</t>
+  </si>
+  <si>
+    <t>Madeena Manzil HOUSE, Perunguzhi, THIRUVANANTHAPURAM, Chirayinkeezhu BLOCK, Chirayinkeezhu PANCHAYATH, Perunguzhi (PO), PIN - 695305</t>
+  </si>
+  <si>
+    <t>BOARD OF KERALA</t>
+  </si>
+  <si>
+    <t>HUMANITIES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +217,12 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -542,7 +572,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -923,17 +953,16 @@
   <dimension ref="A1:L20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="122.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -973,6 +1002,44 @@
       </c>
       <c r="L1" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2">
+        <v>16828</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2">
+        <v>9645184118</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2">
+        <v>9645184118</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -982,6 +1049,12 @@
       <c r="H20" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C100" xr:uid="{311CF363-0780-4854-8806-9AA7017039FD}">
+      <formula1>"TH-1,TH-2,AL-1,AL-2,AL-3,AL-4,Foundation A,Foundation B"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>